<commit_message>
test output foler dlted
</commit_message>
<xml_diff>
--- a/Hero_Hub_UI_Testing/src/test/resources/TestData/ExcelTestData.xlsx
+++ b/Hero_Hub_UI_Testing/src/test/resources/TestData/ExcelTestData.xlsx
@@ -3,6 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Study\Framework\HeroHUbHybridFramework\Hero_Hub_UI_Testing\src\test\resources\TestData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="14520" windowHeight="3340"/>
   </bookViews>
@@ -10,7 +15,6 @@
     <sheet name="0_LoginTest" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -20,13 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>MobileNumber</t>
-  </si>
-  <si>
-    <t>Otp</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Username</t>
   </si>
@@ -34,13 +32,16 @@
     <t>Password</t>
   </si>
   <si>
-    <t>Emergency Number</t>
-  </si>
-  <si>
     <t>Admin</t>
   </si>
   <si>
     <t>admin123</t>
+  </si>
+  <si>
+    <t>Test Scenario</t>
+  </si>
+  <si>
+    <t>Valid</t>
   </si>
 </sst>
 </file>
@@ -106,11 +107,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -393,62 +393,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.453125" customWidth="1"/>
-    <col min="5" max="5" width="15.81640625" customWidth="1"/>
-    <col min="6" max="6" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" customWidth="1"/>
+    <col min="3" max="3" width="14.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
-        <v>7387765344</v>
-      </c>
-      <c r="B2" s="1">
-        <v>7385820122</v>
-      </c>
-      <c r="C2" s="1">
-        <v>123456</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="Automation@11"/>
+    <hyperlink ref="C2" r:id="rId1" display="Automation@11"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>